<commit_message>
Committing Project report under reports folder
</commit_message>
<xml_diff>
--- a/Sales Data Processing and Business Insights System/project/reports/Report.xlsx
+++ b/Sales Data Processing and Business Insights System/project/reports/Report.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sc_BuhleMukhuba_2026\Sales Data Processing and Business Insights System\project\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sc_BuhleMukhuba_2026\Sales Data Processing and Business Insights System\project\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ECDA0C82-8AC0-40A7-8370-F440D38E6126}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4FAEFE5-AEC0-4600-B888-8964243DEC1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{3E2041CA-107C-46DC-9D1D-AC8AD52C858D}"/>
   </bookViews>
@@ -25,9 +25,8 @@
   <calcPr calcId="191029"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId4"/>
-    <pivotCache cacheId="2" r:id="rId5"/>
+    <pivotCache cacheId="1" r:id="rId5"/>
   </pivotCaches>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
       <x14:slicerCaches>
@@ -643,7 +642,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
@@ -653,8 +652,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -702,12 +700,12 @@
   </cellStyles>
   <dxfs count="2">
     <dxf>
+      <numFmt numFmtId="19" formatCode="yyyy/mm/dd"/>
+    </dxf>
+    <dxf>
       <font>
         <color auto="1"/>
       </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="yyyy/mm/dd"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1947,6 +1945,11 @@
                 </a:contourClr>
               </a:sp3d>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-F067-4CE2-8DC2-E1CA91F51E06}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -1970,6 +1973,11 @@
                 </a:contourClr>
               </a:sp3d>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-F067-4CE2-8DC2-E1CA91F51E06}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -1993,6 +2001,11 @@
                 </a:contourClr>
               </a:sp3d>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-F067-4CE2-8DC2-E1CA91F51E06}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="3"/>
@@ -2018,6 +2031,11 @@
                 </a:contourClr>
               </a:sp3d>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-F067-4CE2-8DC2-E1CA91F51E06}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="4"/>
@@ -2043,6 +2061,11 @@
                 </a:contourClr>
               </a:sp3d>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-F067-4CE2-8DC2-E1CA91F51E06}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:spPr>
@@ -3157,6 +3180,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-FFD2-4763-B493-CBEE23DDC870}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:dLbl>
@@ -3225,6 +3253,9 @@
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
                   <c15:showDataLabelsRange val="0"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-FFD2-4763-B493-CBEE23DDC870}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -6401,8 +6432,8 @@
       <xdr:row>24</xdr:row>
       <xdr:rowOff>91965</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="10" name="product">
@@ -6425,7 +6456,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -6603,8 +6634,8 @@
           </a:graphicData>
         </a:graphic>
       </xdr:graphicFrame>
-      <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-        <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+        <mc:Choice Requires="a14">
           <xdr:graphicFrame macro="">
             <xdr:nvGraphicFramePr>
               <xdr:cNvPr id="9" name="region">
@@ -6627,7 +6658,7 @@
             </a:graphic>
           </xdr:graphicFrame>
         </mc:Choice>
-        <mc:Fallback>
+        <mc:Fallback xmlns="">
           <xdr:sp macro="" textlink="">
             <xdr:nvSpPr>
               <xdr:cNvPr id="0" name=""/>
@@ -6666,8 +6697,8 @@
           </xdr:sp>
         </mc:Fallback>
       </mc:AlternateContent>
-      <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-        <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+        <mc:Choice Requires="a14">
           <xdr:graphicFrame macro="">
             <xdr:nvGraphicFramePr>
               <xdr:cNvPr id="12" name="month">
@@ -6690,7 +6721,7 @@
             </a:graphic>
           </xdr:graphicFrame>
         </mc:Choice>
-        <mc:Fallback>
+        <mc:Fallback xmlns="">
           <xdr:sp macro="" textlink="">
             <xdr:nvSpPr>
               <xdr:cNvPr id="0" name=""/>
@@ -7123,11 +7154,95 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>305409</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>33130</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>437488</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>48820</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{40B036E0-EB91-4BE2-BCF1-6609F6DF803C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="835496" y="971826"/>
+          <a:ext cx="1954253" cy="578907"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>457808</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>53008</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>589887</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>68698</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{207BB56E-C612-4C78-9387-0C48725F5814}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14350504" y="991704"/>
+          <a:ext cx="1954253" cy="578907"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8537,452 +8652,6 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BB14BFD8-20AB-4306-91C9-DDA8620A7135}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="E3:F7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0" sortType="descending">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="1">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="5">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of revenue" fld="7" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleMedium2" showRowHeaders="1" showColHeaders="1" showRowStripes="1" showColStripes="1" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AD66994A-D681-4A33-8AFB-B4704C5BE76E}" name="Sales by region" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8">
-  <location ref="A3:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0">
-      <items count="51">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="21"/>
-        <item x="22"/>
-        <item x="23"/>
-        <item x="24"/>
-        <item x="25"/>
-        <item x="26"/>
-        <item x="27"/>
-        <item x="28"/>
-        <item x="29"/>
-        <item x="30"/>
-        <item x="31"/>
-        <item x="32"/>
-        <item x="33"/>
-        <item x="34"/>
-        <item x="35"/>
-        <item x="36"/>
-        <item x="37"/>
-        <item x="38"/>
-        <item x="39"/>
-        <item x="40"/>
-        <item x="41"/>
-        <item x="42"/>
-        <item x="43"/>
-        <item x="44"/>
-        <item x="45"/>
-        <item x="46"/>
-        <item x="47"/>
-        <item x="48"/>
-        <item x="49"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="3"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="8"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of revenue" fld="7" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="6" name="date">
-      <autoFilter ref="A1">
-        <filterColumn colId="0">
-          <customFilters and="1">
-            <customFilter operator="greaterThanOrEqual" val="45323"/>
-            <customFilter operator="lessThanOrEqual" val="45412"/>
-          </customFilters>
-        </filterColumn>
-      </autoFilter>
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{0605FD5F-26C8-4aeb-8148-2DB25E43C511}">
-          <x15:pivotFilter useWholeDay="1"/>
-        </ext>
-      </extLst>
-    </filter>
-  </filters>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable11.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7859CB44-A862-4CA5-BE15-CFD0A306794F}" name="Quantity" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A34:A35" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="3"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0">
-      <items count="8">
-        <item x="3"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item x="5"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="5">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of quantity" fld="5" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="0">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8630491F-F08B-49F1-940F-97948256AC3A}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A11:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="3"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="5">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of revenue" fld="7" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleMedium2" showRowHeaders="1" showColHeaders="1" showRowStripes="1" showColStripes="1" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{52A30C47-CBBD-4014-8FB4-D1E3DC34AC99}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="8"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of revenue" fld="7" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleMedium2" showRowHeaders="1" showColHeaders="1" showRowStripes="1" showColStripes="1" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D4F61047-0585-45D2-925F-ABCB178E6C44}" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E11:F16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
@@ -9061,176 +8730,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FE1C5BED-0277-4E27-9603-4B6AE4EFD2CC}" name="Revenue" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A31:A32" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="3"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="5">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of revenue" fld="7" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6BC83E6F-4AE7-4A5F-AC8E-5917ED0E2C89}" name="Salesperson performance" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
-  <location ref="A24:B29" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="3"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="5">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="9"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of revenue" fld="7" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{014C6A68-B203-401E-AE86-8D5CF87BC2AE}" name="product category dis" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="23">
+<file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{014C6A68-B203-401E-AE86-8D5CF87BC2AE}" name="product category dis" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="23">
   <location ref="A15:B22" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
@@ -9424,8 +8925,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2150134B-82E8-4471-BAF3-55481DDA2BDA}" name="Monthly Revenue" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
+<file path=xl/pivotTables/pivotTable11.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2150134B-82E8-4471-BAF3-55481DDA2BDA}" name="Monthly Revenue" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
   <location ref="A9:B13" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
@@ -9510,8 +9011,211 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C337CFC0-671E-4BAE-B119-173E217D49EF}" name="Units per salesperson" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12">
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BB14BFD8-20AB-4306-91C9-DDA8620A7135}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="E3:F7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of revenue" fld="7" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleMedium2" showRowHeaders="1" showColHeaders="1" showRowStripes="1" showColStripes="1" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8630491F-F08B-49F1-940F-97948256AC3A}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A11:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="3"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of revenue" fld="7" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleMedium2" showRowHeaders="1" showColHeaders="1" showRowStripes="1" showColStripes="1" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{52A30C47-CBBD-4014-8FB4-D1E3DC34AC99}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="8"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of revenue" fld="7" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleMedium2" showRowHeaders="1" showColHeaders="1" showRowStripes="1" showColStripes="1" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C337CFC0-671E-4BAE-B119-173E217D49EF}" name="Units per salesperson" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12">
   <location ref="A37:B42" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
@@ -9620,6 +9324,417 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AD66994A-D681-4A33-8AFB-B4704C5BE76E}" name="Sales by region" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8">
+  <location ref="A3:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="51">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item x="30"/>
+        <item x="31"/>
+        <item x="32"/>
+        <item x="33"/>
+        <item x="34"/>
+        <item x="35"/>
+        <item x="36"/>
+        <item x="37"/>
+        <item x="38"/>
+        <item x="39"/>
+        <item x="40"/>
+        <item x="41"/>
+        <item x="42"/>
+        <item x="43"/>
+        <item x="44"/>
+        <item x="45"/>
+        <item x="46"/>
+        <item x="47"/>
+        <item x="48"/>
+        <item x="49"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="3"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="8"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of revenue" fld="7" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <filters count="1">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="6" name="date">
+      <autoFilter ref="A1">
+        <filterColumn colId="0">
+          <customFilters and="1">
+            <customFilter operator="greaterThanOrEqual" val="45323"/>
+            <customFilter operator="lessThanOrEqual" val="45412"/>
+          </customFilters>
+        </filterColumn>
+      </autoFilter>
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{0605FD5F-26C8-4aeb-8148-2DB25E43C511}">
+          <x15:pivotFilter useWholeDay="1"/>
+        </ext>
+      </extLst>
+    </filter>
+  </filters>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FE1C5BED-0277-4E27-9603-4B6AE4EFD2CC}" name="Revenue" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A31:A32" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="3"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of revenue" fld="7" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6BC83E6F-4AE7-4A5F-AC8E-5917ED0E2C89}" name="Salesperson performance" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
+  <location ref="A24:B29" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="3"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="9"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of revenue" fld="7" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7859CB44-A862-4CA5-BE15-CFD0A306794F}" name="Quantity" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A34:A35" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="3"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0">
+      <items count="8">
+        <item x="3"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="5"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of quantity" fld="5" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="1">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
 <slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_region" xr10:uid="{B7835F11-A822-40C3-B18B-76D3FBA9DC43}" sourceName="region">
   <pivotTables>
@@ -9704,7 +9819,7 @@
   <autoFilter ref="A1:J51" xr:uid="{0EDEA3D0-C3E2-4CE6-A2D6-D24F9209B1B8}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{03CB79EB-8710-4778-A901-ACDB48783752}" name="transaction_id"/>
-    <tableColumn id="2" xr3:uid="{BA986633-A9E7-4DDF-A46D-6D5769612935}" name="date" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{BA986633-A9E7-4DDF-A46D-6D5769612935}" name="date" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{FEFDA565-EF7B-4539-9808-A39777303903}" name="month"/>
     <tableColumn id="4" xr3:uid="{F1117D6A-1157-4BF4-9684-3DE874B8A623}" name="product"/>
     <tableColumn id="5" xr3:uid="{296DD317-742E-462D-ACB2-916A2EACA303}" name="category"/>
@@ -10209,7 +10324,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A3:D42"/>
+  <dimension ref="A3:C42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="0" hidden="1" customWidth="1"/>
@@ -10230,7 +10345,7 @@
       <c r="A4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4">
         <v>270000</v>
       </c>
     </row>
@@ -10238,7 +10353,7 @@
       <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5">
         <v>260500</v>
       </c>
     </row>
@@ -10246,7 +10361,7 @@
       <c r="A6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6">
         <v>225000</v>
       </c>
     </row>
@@ -10254,7 +10369,7 @@
       <c r="A7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7">
         <v>157000</v>
       </c>
     </row>
@@ -10270,7 +10385,7 @@
       <c r="A10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10">
         <v>164500</v>
       </c>
     </row>
@@ -10278,7 +10393,7 @@
       <c r="A11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11">
         <v>200500</v>
       </c>
     </row>
@@ -10286,7 +10401,7 @@
       <c r="A12" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12">
         <v>271500</v>
       </c>
     </row>
@@ -10294,7 +10409,7 @@
       <c r="A13" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13">
         <v>276000</v>
       </c>
     </row>
@@ -10310,7 +10425,7 @@
       <c r="A16" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="5">
+      <c r="B16">
         <v>770000</v>
       </c>
     </row>
@@ -10318,7 +10433,7 @@
       <c r="A17" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="5">
+      <c r="B17">
         <v>440000</v>
       </c>
     </row>
@@ -10326,7 +10441,7 @@
       <c r="A18" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="5">
+      <c r="B18">
         <v>180000</v>
       </c>
     </row>
@@ -10334,7 +10449,7 @@
       <c r="A19" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="5">
+      <c r="B19">
         <v>150000</v>
       </c>
     </row>
@@ -10342,7 +10457,7 @@
       <c r="A20" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="5">
+      <c r="B20">
         <v>142500</v>
       </c>
     </row>
@@ -10350,7 +10465,7 @@
       <c r="A21" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="5">
+      <c r="B21">
         <v>75000</v>
       </c>
     </row>
@@ -10358,7 +10473,7 @@
       <c r="A22" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="5">
+      <c r="B22">
         <v>67500</v>
       </c>
     </row>
@@ -10374,7 +10489,7 @@
       <c r="A25" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B25" s="5">
+      <c r="B25">
         <v>270000</v>
       </c>
     </row>
@@ -10382,7 +10497,7 @@
       <c r="A26" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B26" s="5">
+      <c r="B26">
         <v>260500</v>
       </c>
     </row>
@@ -10390,7 +10505,7 @@
       <c r="A27" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B27" s="5">
+      <c r="B27">
         <v>204000</v>
       </c>
     </row>
@@ -10398,7 +10513,7 @@
       <c r="A28" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B28" s="5">
+      <c r="B28">
         <v>157000</v>
       </c>
     </row>
@@ -10406,7 +10521,7 @@
       <c r="A29" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="5">
+      <c r="B29">
         <v>21000</v>
       </c>
     </row>
@@ -10416,7 +10531,7 @@
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A32" s="5">
+      <c r="A32">
         <v>912500</v>
       </c>
     </row>
@@ -10426,7 +10541,7 @@
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" s="6">
+      <c r="A35" s="5">
         <v>165</v>
       </c>
     </row>
@@ -10442,7 +10557,7 @@
       <c r="A38" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B38" s="5">
+      <c r="B38">
         <v>43</v>
       </c>
     </row>
@@ -10450,7 +10565,7 @@
       <c r="A39" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B39" s="5">
+      <c r="B39">
         <v>47</v>
       </c>
     </row>
@@ -10458,7 +10573,7 @@
       <c r="A40" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B40" s="5">
+      <c r="B40">
         <v>39</v>
       </c>
     </row>
@@ -10466,7 +10581,7 @@
       <c r="A41" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B41" s="5">
+      <c r="B41">
         <v>32</v>
       </c>
     </row>
@@ -10474,7 +10589,7 @@
       <c r="A42" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B42" s="5">
+      <c r="B42">
         <v>4</v>
       </c>
     </row>

</xml_diff>